<commit_message>
feat(onboarding): persist investor KYC on initial setup submit
</commit_message>
<xml_diff>
--- a/ARL_Test_Tracker.xlsx
+++ b/ARL_Test_Tracker.xlsx
@@ -11966,17 +11966,17 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>3-step onboarding wizard (personal / KYC / bank). Client-side only — no backend submission; final step shows snackbar confirmation only. Backend onboard endpoint not wired in.</t>
+          <t>3-step wizard now persists on submit via InvestorRepository.upsertOnboarding -&gt; investors row keyed to auth.uid(). Validators: PAN ^[A-Z]{5}[0-9]{4}[A-Z]$, Aadhaar 12 digits, IFSC ^[A-Z]{4}0[A-Z0-9]{6}$, account 9-18 digits, DOB DD-MM-YYYY not in future, email regex. Inline errors via TextFormField + AutovalidateMode.onUserInteraction. PAN/Aadhaar/account stored as masked tail only - full numbers never reach DB. Migration 027: INSERT + UPDATE RLS for own row, GRANT to authenticated, arl_id nullable. Submit -&gt; snackbar + go(home). Analyzer clean.</t>
         </is>
       </c>
       <c r="E8" s="22" t="inlineStr">
         <is>
-          <t>From /auth tap 'Get Started' → /setup. Wizard steps: (1) name+email+DOB, (2) PAN+Aadhaar, (3) bank account+IFSC. Each step has Next button. Final 'Submit' shows 'Setup submitted' snackbar and routes to /. Data not persisted to investors table.</t>
+          <t>From /auth tap 'Get Started' -&gt; /setup. Step 1 collects full name, email (pre-filled from auth user), DOB; Continue validates inline. Step 2 collects PAN (auto-uppercased) + Aadhaar (digits only, max 12). Step 3 collects bank name, IFSC, account, holder name. Submit shows spinner, calls upsertOnboarding which writes id, name, email, kyc_status='pending', date_of_birth, plus masked pan/aadhaar/account, bank_name, bank_ifsc, bank_holder_name. Success -&gt; currentInvestorProvider invalidated, snackbar, go(home).</t>
         </is>
       </c>
       <c r="F8" s="22" t="inlineStr">

</xml_diff>

<commit_message>
feat(explore): persist consultation requests
</commit_message>
<xml_diff>
--- a/ARL_Test_Tracker.xlsx
+++ b/ARL_Test_Tracker.xlsx
@@ -12304,17 +12304,17 @@
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>Routed at /explore. marketplaceProjectsProvider queries projects WHERE is_listed_in_marketplace=true (live). Filter pills + project picker + unit slider work. 'Request Consultation' button is a STUB (snackbar only, TODO comment in code; no support_repository call).</t>
+          <t>'Request Consultation' CTA now writes a row to consultation_requests via ConsultationRequestsRepository (RLS scoped to auth.uid()). Button shows a spinner and is disabled in-flight; 24h dedup check first - if the same user has an open 'new' request for this project within 24h, no duplicate insert is made and the toast says we already have the request. Migration 028 adds the table + RLS + indexes. Analyzer clean.</t>
         </is>
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>Tap Explore in bottom nav. Sees filter pills (All / Open for Reservation / Coming Soon). Selects a marketplace project from dropdown → detail card (crop, tier, available units, price). Slider adjusts unit count → total cost + projected return update live. 'Request Consultation' button → snackbar 'Request received' but nothing persisted.</t>
+          <t>Tap Explore in bottom nav -&gt; filter pills + grid of marketplace projects. Open one, choose unit count via slider/custom input, then tap 'Request Consultation'. Button swaps for an inline spinner, ConsultationRequestsRepository.createConsultation runs the 24h dedup query, then either inserts a new row or returns the existing one. Toast confirms the submission. Subsequent taps within 24h surface the friendly 'already requested' message instead of duplicating.</t>
         </is>
       </c>
       <c r="F18" s="22" t="inlineStr">

</xml_diff>

<commit_message>
feat(exit): persist exit requests with duplicate guard
</commit_message>
<xml_diff>
--- a/ARL_Test_Tracker.xlsx
+++ b/ARL_Test_Tracker.xlsx
@@ -12656,17 +12656,17 @@
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D29" s="26" t="inlineStr">
         <is>
-          <t>Routed at /exit. _earliestInvestmentDateProvider queries investor_units for earliest investment_date (real Supabase, 5-sec session wait). 'Request Exit' button is a STUB — no backend persistence.</t>
+          <t>'Request Exit' CTA now opens a reason dialog and writes to exit_requests via ExitRequestsRepository (RLS scoped to auth.uid()). FK is investor_unit_id pulled from the earliest investor_units row. DB-level partial unique index (investor_unit_id WHERE status='pending') is the race-safe dedup; client catches Postgrest 23505 and surfaces the existing pending row. After submit the screen flips to a 'pending review' card with the submission date - the CTA is no longer shown until staff moves status off pending. Migration 029. Analyzer clean.</t>
         </is>
       </c>
       <c r="E29" s="26" t="inlineStr">
         <is>
-          <t>From Profile tap 'Project Exit' → /exit. Shows investment date, lock-in end date (investment + 5y), time remaining. If lock-in passed → 'Request Exit' button enabled; tap shows snackbar 'Exit request submitted. Our team will review within 5 business days' but no row is created. If not eligible → disabled grey button with lock icon. 'Learn about the exit process →' shows mock multiline snackbar.</t>
+          <t>From Profile tap 'Project Exit' -&gt; /exit. Sees investment date, lock-in end date, eligibility chip (locked yellow vs eligible green). If a pending exit_request already exists for the earliest investor_unit, the bottom card shows 'Exit request pending review' with the submission date and the CTA is hidden. Otherwise the CTA is enabled iff the lock-in has passed; tapping opens a reason dialog (3-line text, optional). Submit shows a spinner, posts to exit_requests with status='pending', invalidates the pending provider, snackbar confirms - card flips to the submitted state.</t>
         </is>
       </c>
       <c r="F29" s="26" t="inlineStr">

</xml_diff>

<commit_message>
docs(ops): document Sec/Bio/Onboarding/Consultation/Exit additions
</commit_message>
<xml_diff>
--- a/ARL_Test_Tracker.xlsx
+++ b/ARL_Test_Tracker.xlsx
@@ -11971,7 +11971,7 @@
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>3-step wizard now persists on submit via InvestorRepository.upsertOnboarding -&gt; investors row keyed to auth.uid(). Validators: PAN ^[A-Z]{5}[0-9]{4}[A-Z]$, Aadhaar 12 digits, IFSC ^[A-Z]{4}0[A-Z0-9]{6}$, account 9-18 digits, DOB DD-MM-YYYY not in future, email regex. Inline errors via TextFormField + AutovalidateMode.onUserInteraction. PAN/Aadhaar/account stored as masked tail only - full numbers never reach DB. Migration 027: INSERT + UPDATE RLS for own row, GRANT to authenticated, arl_id nullable. Submit -&gt; snackbar + go(home). Analyzer clean.</t>
+          <t>3-step wizard now persists on submit via InvestorRepository.upsertOnboarding -&gt; investors row keyed to auth.uid(). Validators: PAN ^[A-Z]{5}[0-9]{4}[A-Z]$, Aadhaar 12 digits, IFSC ^[A-Z]{4}0[A-Z0-9]{6}$, account 9-18 digits, DOB DD-MM-YYYY not in future, email regex. Inline errors via TextFormField + AutovalidateMode.onUserInteraction. PAN/Aadhaar/account stored as masked tail only - full numbers never reach DB. Migration 027: INSERT + UPDATE RLS for own row, GRANT to authenticated, arl_id nullable. Submit -&gt; snackbar + go(home). Analyzer clean. Documented in ops_admin_guide.md §6.3 Investor self-onboarding (InitialSetupScreen).</t>
         </is>
       </c>
       <c r="E8" s="22" t="inlineStr">
@@ -12012,7 +12012,7 @@
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>Registered at /biometric outside the ShellRoute (full-screen, no bottom nav). Pops with bool result: true on biometric success, false on cancel. Reached as an enrollment gate from SecurityScreen when the Biometric Login toggle is turned on; the persisted biometric_enabled flag flips only after a real BiometricGuard check passes. Legacy direct-entry path still routes to home on success. Analyzer clean.</t>
+          <t>Registered at /biometric outside the ShellRoute (full-screen, no bottom nav). Pops with bool result: true on biometric success, false on cancel. Reached as an enrollment gate from SecurityScreen when the Biometric Login toggle is turned on; the persisted biometric_enabled flag flips only after a real BiometricGuard check passes. Legacy direct-entry path still routes to home on success. Analyzer clean. Documented in ops_admin_guide.md §6.2 Biometric enrollment gate (BiometricScreen).</t>
         </is>
       </c>
       <c r="E9" s="26" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>'Request Consultation' CTA now writes a row to consultation_requests via ConsultationRequestsRepository (RLS scoped to auth.uid()). Button shows a spinner and is disabled in-flight; 24h dedup check first - if the same user has an open 'new' request for this project within 24h, no duplicate insert is made and the toast says we already have the request. Migration 028 adds the table + RLS + indexes. Analyzer clean.</t>
+          <t>'Request Consultation' CTA now writes a row to consultation_requests via ConsultationRequestsRepository (RLS scoped to auth.uid()). Button shows a spinner and is disabled in-flight; 24h dedup check first - if the same user has an open 'new' request for this project within 24h, no duplicate insert is made and the toast says we already have the request. Migration 028 adds the table + RLS + indexes. Analyzer clean. Documented in ops_admin_guide.md §6.4 Consultation requests (ExploreScreen).</t>
         </is>
       </c>
       <c r="E18" s="22" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="D25" s="26" t="inlineStr">
         <is>
-          <t>Toggles (biometric, notifications) persist to user_settings via UserSettingsRepository on Supabase (RLS-scoped to auth.uid). App PIN: set/change/remove flow stores salted client-side SHA-256 iterated hash (never plaintext) keyed off auth user. Last-login + login history rendered from login_events table written on every AuthChangeEvent.signedIn. Migration 026 adds user_settings + login_events with RLS. Analyzer clean.</t>
+          <t>Toggles (biometric, notifications) persist to user_settings via UserSettingsRepository on Supabase (RLS-scoped to auth.uid). App PIN: set/change/remove flow stores salted client-side SHA-256 iterated hash (never plaintext) keyed off auth user. Last-login + login history rendered from login_events table written on every AuthChangeEvent.signedIn. Migration 026 adds user_settings + login_events with RLS. Analyzer clean. Documented in ops_admin_guide.md §6.1 Security &amp; PIN (SecurityScreen).</t>
         </is>
       </c>
       <c r="E25" s="26" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="D29" s="26" t="inlineStr">
         <is>
-          <t>'Request Exit' CTA now opens a reason dialog and writes to exit_requests via ExitRequestsRepository (RLS scoped to auth.uid()). FK is investor_unit_id pulled from the earliest investor_units row. DB-level partial unique index (investor_unit_id WHERE status='pending') is the race-safe dedup; client catches Postgrest 23505 and surfaces the existing pending row. After submit the screen flips to a 'pending review' card with the submission date - the CTA is no longer shown until staff moves status off pending. Migration 029. Analyzer clean.</t>
+          <t>'Request Exit' CTA now opens a reason dialog and writes to exit_requests via ExitRequestsRepository (RLS scoped to auth.uid()). FK is investor_unit_id pulled from the earliest investor_units row. DB-level partial unique index (investor_unit_id WHERE status='pending') is the race-safe dedup; client catches Postgrest 23505 and surfaces the existing pending row. After submit the screen flips to a 'pending review' card with the submission date - the CTA is no longer shown until staff moves status off pending. Migration 029. Analyzer clean. Documented in ops_admin_guide.md §6.5 Exit requests (ExitScreen).</t>
         </is>
       </c>
       <c r="E29" s="26" t="inlineStr">

</xml_diff>